<commit_message>
Added RegisterTest, ConfigReader, ExtentReports and Screenshot
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/logindata.xlsx
+++ b/src/main/resources/testdata/logindata.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="RegisterData" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="LoginData" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,7 +12,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
+  <si>
+    <t>name</t>
+  </si>
   <si>
     <t>email</t>
   </si>
@@ -19,7 +23,82 @@
     <t>password</t>
   </si>
   <si>
+    <t>firstname</t>
+  </si>
+  <si>
+    <t>last name</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>state</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>zipcode</t>
+  </si>
+  <si>
+    <t>mobile</t>
+  </si>
+  <si>
     <t>testcase</t>
+  </si>
+  <si>
+    <t>Bhargavi Test</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>bhargavi_test1@gmail.com</t>
+    </r>
+  </si>
+  <si>
+    <t>Test@123</t>
+  </si>
+  <si>
+    <t>bhargavi</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>near maszid road , chennai</t>
+  </si>
+  <si>
+    <t>tamilandu</t>
+  </si>
+  <si>
+    <t>chennai</t>
+  </si>
+  <si>
+    <t>Valid Registrati</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>bhargavi_test2@gmail.com</t>
+    </r>
+  </si>
+  <si>
+    <t>hsr layout</t>
+  </si>
+  <si>
+    <t>karnataka</t>
+  </si>
+  <si>
+    <t>mangalore</t>
+  </si>
+  <si>
+    <t>Missing Name</t>
   </si>
   <si>
     <r>
@@ -29,9 +108,6 @@
       </rPr>
       <t>kotianbs4@gmail.com</t>
     </r>
-  </si>
-  <si>
-    <t>Test@123</t>
   </si>
   <si>
     <t>Valid Login</t>
@@ -82,13 +158,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <color rgb="FF0000FF"/>
-    </font>
-    <font>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
   </fonts>
   <fills count="2">
@@ -127,6 +203,10 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -334,6 +414,10 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="17.38"/>
+    <col customWidth="1" min="4" max="6" width="29.5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -345,38 +429,157 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>5</v>
+        <v>12</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="2">
+        <v>678456.0</v>
+      </c>
+      <c r="J2" s="2">
+        <v>9.999999999E9</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="s">
-        <v>6</v>
-      </c>
       <c r="B3" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>7</v>
+        <v>20</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="2">
+        <v>666345.0</v>
+      </c>
+      <c r="J3" s="2">
+        <v>8.888888888E9</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="B2"/>
+    <hyperlink r:id="rId2" ref="B3"/>
+  </hyperlinks>
+  <drawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="24.13"/>
+    <col customWidth="1" min="2" max="2" width="33.13"/>
+    <col customWidth="1" min="3" max="3" width="22.88"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>10</v>
+      <c r="A4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>